<commit_message>
Add table loops, display fields, and GitHub Pages for examples.
Ship repeating-table bind/preview, BASE_URL-safe template assets, and an Actions workflow that publishes native/custom demos.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/custom-ui/public/templates/采购合同.xlsx
+++ b/examples/custom-ui/public/templates/采购合同.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>采购合同</t>
   </si>
@@ -67,83 +67,95 @@
     <t>{{partyBContact}}</t>
   </si>
   <si>
+    <t>合同金额（元）</t>
+  </si>
+  <si>
+    <t>{{amount:number}}</t>
+  </si>
+  <si>
+    <t>付款方式</t>
+  </si>
+  <si>
+    <t>{{payMethod:select}}</t>
+  </si>
+  <si>
+    <t>付款期限</t>
+  </si>
+  <si>
+    <t>{{payTerm}}</t>
+  </si>
+  <si>
+    <t>交货日期</t>
+  </si>
+  <si>
+    <t>{{deliveryDate:date}}</t>
+  </si>
+  <si>
+    <t>交货地点</t>
+  </si>
+  <si>
+    <t>{{deliveryPlace}}</t>
+  </si>
+  <si>
+    <t>质保期限</t>
+  </si>
+  <si>
+    <t>{{warranty}}</t>
+  </si>
+  <si>
+    <t>签订日期</t>
+  </si>
+  <si>
+    <t>{{signDate:date}}</t>
+  </si>
+  <si>
+    <t>备注说明</t>
+  </si>
+  <si>
+    <t>{{note:textarea}}</t>
+  </si>
+  <si>
+    <t>填写日</t>
+  </si>
+  <si>
+    <t>{{filledAt:display}}</t>
+  </si>
+  <si>
+    <t>序号</t>
+  </si>
+  <si>
     <t>货物名称</t>
   </si>
   <si>
-    <t>{{goods}}</t>
-  </si>
-  <si>
     <t>规格型号</t>
   </si>
   <si>
-    <t>{{spec}}</t>
-  </si>
-  <si>
     <t>数量</t>
   </si>
   <si>
-    <t>{{qty:number}}</t>
-  </si>
-  <si>
-    <t>单价（元）</t>
-  </si>
-  <si>
-    <t>{{unitPrice:number}}</t>
-  </si>
-  <si>
-    <t>合同金额（元）</t>
-  </si>
-  <si>
-    <t>{{amount:number}}</t>
-  </si>
-  <si>
-    <t>付款方式</t>
-  </si>
-  <si>
-    <t>{{payMethod:select}}</t>
-  </si>
-  <si>
-    <t>付款期限</t>
-  </si>
-  <si>
-    <t>{{payTerm}}</t>
-  </si>
-  <si>
-    <t>交货日期</t>
-  </si>
-  <si>
-    <t>{{deliveryDate:date}}</t>
-  </si>
-  <si>
-    <t>交货地点</t>
-  </si>
-  <si>
-    <t>{{deliveryPlace}}</t>
-  </si>
-  <si>
-    <t>质保期限</t>
-  </si>
-  <si>
-    <t>{{warranty}}</t>
-  </si>
-  <si>
-    <t>签订日期</t>
-  </si>
-  <si>
-    <t>{{signDate:date}}</t>
-  </si>
-  <si>
-    <t>备注说明</t>
-  </si>
-  <si>
-    <t>{{note:textarea}}</t>
+    <t>单价</t>
+  </si>
+  <si>
+    <t>{{items.$index}}</t>
+  </si>
+  <si>
+    <t>{{items.name}}</t>
+  </si>
+  <si>
+    <t>{{items.spec}}</t>
+  </si>
+  <si>
+    <t>{{items.qty:number}}</t>
+  </si>
+  <si>
+    <t>{{items.unitPrice:number}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -165,6 +177,10 @@
     <font>
       <b/>
       <color rgb="FF1B3A5C"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -222,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -233,6 +249,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,10 +593,11 @@
   <sheetPr>
     <tabColor rgb="FF1B3A5C"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="18" customWidth="1"/>
+    <col min="1" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -767,38 +786,42 @@
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="C22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="D22" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="E22" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="5" t="s">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
+      <c r="B23" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>45</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="19">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B4:D4"/>
@@ -818,9 +841,6 @@
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>